<commit_message>
Suivi : iterations 3 et 4 marquees dans l explosion du projet
72 fonctionnalites MVP realisees, 8 partielles

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Explosion du projet - MAJ.xlsx
+++ b/docs/Explosion du projet - MAJ.xlsx
@@ -1774,9 +1774,14 @@
           <t>Haute</t>
         </is>
       </c>
-      <c r="F19" s="2" t="inlineStr">
-        <is>
-          <t>À faire</t>
+      <c r="F19" s="33" t="inlineStr">
+        <is>
+          <t>✅ Réalisé</t>
+        </is>
+      </c>
+      <c r="G19" s="34" t="inlineStr">
+        <is>
+          <t>Itération 4 — liste + détail</t>
         </is>
       </c>
     </row>
@@ -1804,9 +1809,14 @@
           <t>Haute</t>
         </is>
       </c>
-      <c r="F20" s="2" t="inlineStr">
-        <is>
-          <t>À faire</t>
+      <c r="F20" s="35" t="inlineStr">
+        <is>
+          <t>🟡 Partiel</t>
+        </is>
+      </c>
+      <c r="G20" s="34" t="inlineStr">
+        <is>
+          <t>Statuts visibles ; transitions avec Escrow/Livraison</t>
         </is>
       </c>
     </row>
@@ -1984,9 +1994,14 @@
           <t>Haute</t>
         </is>
       </c>
-      <c r="F26" s="2" t="inlineStr">
-        <is>
-          <t>À faire</t>
+      <c r="F26" s="35" t="inlineStr">
+        <is>
+          <t>🟡 Partiel</t>
+        </is>
+      </c>
+      <c r="G26" s="34" t="inlineStr">
+        <is>
+          <t>Liste visible ; traitement avec Escrow</t>
         </is>
       </c>
     </row>
@@ -2830,7 +2845,7 @@
       </c>
       <c r="G53" s="34" t="inlineStr">
         <is>
-          <t>Itération 3</t>
+          <t>Itération 3 — 8 catégories</t>
         </is>
       </c>
     </row>
@@ -2865,7 +2880,7 @@
       </c>
       <c r="G54" s="34" t="inlineStr">
         <is>
-          <t>Itération 3</t>
+          <t>Itération 3 — 30 sous-catégories</t>
         </is>
       </c>
     </row>
@@ -2935,7 +2950,7 @@
       </c>
       <c r="G56" s="34" t="inlineStr">
         <is>
-          <t>Itération 3 — contrôle client et serveur</t>
+          <t>Itération 3 — validé client et serveur</t>
         </is>
       </c>
     </row>
@@ -3005,7 +3020,7 @@
       </c>
       <c r="G58" s="34" t="inlineStr">
         <is>
-          <t>Itération 3 — réordonnancement dans le formulaire</t>
+          <t>Itération 3 — réorganisable</t>
         </is>
       </c>
     </row>
@@ -3105,7 +3120,7 @@
       </c>
       <c r="G61" s="34" t="inlineStr">
         <is>
-          <t>Itération 3 — fichiers Storage nettoyés</t>
+          <t>Itération 3</t>
         </is>
       </c>
     </row>
@@ -3140,7 +3155,7 @@
       </c>
       <c r="G62" s="34" t="inlineStr">
         <is>
-          <t>Itération 3</t>
+          <t>Itération 3 — FCFA entiers</t>
         </is>
       </c>
     </row>
@@ -3175,7 +3190,7 @@
       </c>
       <c r="G63" s="34" t="inlineStr">
         <is>
-          <t>Un seul palier pour l'instant (prix de gros)</t>
+          <t>Un palier (prix de gros) ; paliers multiples à venir</t>
         </is>
       </c>
     </row>
@@ -3210,7 +3225,7 @@
       </c>
       <c r="G64" s="34" t="inlineStr">
         <is>
-          <t>Itération 3 — prix + quantité minimum</t>
+          <t>Itération 3 — appliqué auto selon quantité</t>
         </is>
       </c>
     </row>
@@ -3350,7 +3365,7 @@
       </c>
       <c r="G68" s="34" t="inlineStr">
         <is>
-          <t>Itération 3 — badge rupture automatique</t>
+          <t>Itération 3 — badge rupture</t>
         </is>
       </c>
     </row>
@@ -3550,7 +3565,7 @@
       </c>
       <c r="G74" s="34" t="inlineStr">
         <is>
-          <t>Itération 3 — brouillon / en ligne</t>
+          <t>Itération 3 — brouillon/en ligne</t>
         </is>
       </c>
     </row>
@@ -3585,7 +3600,7 @@
       </c>
       <c r="G75" s="34" t="inlineStr">
         <is>
-          <t>Itération 3</t>
+          <t>Itération 3 — photos purgées du Storage</t>
         </is>
       </c>
     </row>
@@ -3632,7 +3647,7 @@
       </c>
       <c r="G77" s="34" t="inlineStr">
         <is>
-          <t>Itération 3 — catégories + nouveautés</t>
+          <t>Itération 3 — hero, catégories, nouveautés</t>
         </is>
       </c>
     </row>
@@ -3702,7 +3717,7 @@
       </c>
       <c r="G79" s="34" t="inlineStr">
         <is>
-          <t>Itération 3 — 8 catégories, 30 sous-catégories</t>
+          <t>Itération 3</t>
         </is>
       </c>
     </row>
@@ -3772,7 +3787,7 @@
       </c>
       <c r="G81" s="34" t="inlineStr">
         <is>
-          <t>Itération 3 — 12 produits par page</t>
+          <t>Itération 3 — 12/page</t>
         </is>
       </c>
     </row>
@@ -3842,7 +3857,7 @@
       </c>
       <c r="G83" s="34" t="inlineStr">
         <is>
-          <t>Itération 3 — titre et description</t>
+          <t>Itération 3 — titre + description</t>
         </is>
       </c>
     </row>
@@ -3982,7 +3997,7 @@
       </c>
       <c r="G87" s="34" t="inlineStr">
         <is>
-          <t>Itération 3 — tri par défaut : plus récents</t>
+          <t>Itération 3 — plus récents par défaut</t>
         </is>
       </c>
     </row>
@@ -4127,9 +4142,14 @@
           <t>Haute</t>
         </is>
       </c>
-      <c r="F92" s="2" t="inlineStr">
-        <is>
-          <t>À faire</t>
+      <c r="F92" s="33" t="inlineStr">
+        <is>
+          <t>✅ Réalisé</t>
+        </is>
+      </c>
+      <c r="G92" s="34" t="inlineStr">
+        <is>
+          <t>Itération 4</t>
         </is>
       </c>
     </row>
@@ -4157,9 +4177,14 @@
           <t>Haute</t>
         </is>
       </c>
-      <c r="F93" s="2" t="inlineStr">
-        <is>
-          <t>À faire</t>
+      <c r="F93" s="33" t="inlineStr">
+        <is>
+          <t>✅ Réalisé</t>
+        </is>
+      </c>
+      <c r="G93" s="34" t="inlineStr">
+        <is>
+          <t>Itération 4 — bornes stock/qté min</t>
         </is>
       </c>
     </row>
@@ -4187,9 +4212,14 @@
           <t>Haute</t>
         </is>
       </c>
-      <c r="F94" s="2" t="inlineStr">
-        <is>
-          <t>À faire</t>
+      <c r="F94" s="33" t="inlineStr">
+        <is>
+          <t>✅ Réalisé</t>
+        </is>
+      </c>
+      <c r="G94" s="34" t="inlineStr">
+        <is>
+          <t>Itération 4</t>
         </is>
       </c>
     </row>
@@ -4217,9 +4247,14 @@
           <t>Haute</t>
         </is>
       </c>
-      <c r="F95" s="2" t="inlineStr">
-        <is>
-          <t>À faire</t>
+      <c r="F95" s="33" t="inlineStr">
+        <is>
+          <t>✅ Réalisé</t>
+        </is>
+      </c>
+      <c r="G95" s="34" t="inlineStr">
+        <is>
+          <t>Itération 4</t>
         </is>
       </c>
     </row>
@@ -4247,9 +4282,14 @@
           <t>Haute</t>
         </is>
       </c>
-      <c r="F96" s="2" t="inlineStr">
-        <is>
-          <t>À faire</t>
+      <c r="F96" s="33" t="inlineStr">
+        <is>
+          <t>✅ Réalisé</t>
+        </is>
+      </c>
+      <c r="G96" s="34" t="inlineStr">
+        <is>
+          <t>Itération 4 — panier groupé par vendeur</t>
         </is>
       </c>
     </row>
@@ -4277,9 +4317,14 @@
           <t>Haute</t>
         </is>
       </c>
-      <c r="F97" s="2" t="inlineStr">
-        <is>
-          <t>À faire</t>
+      <c r="F97" s="33" t="inlineStr">
+        <is>
+          <t>✅ Réalisé</t>
+        </is>
+      </c>
+      <c r="G97" s="34" t="inlineStr">
+        <is>
+          <t>Itération 4 — forfait provisoire 1 000 FCFA/vendeur</t>
         </is>
       </c>
     </row>
@@ -4307,9 +4352,14 @@
           <t>Moyenne</t>
         </is>
       </c>
-      <c r="F98" s="2" t="inlineStr">
-        <is>
-          <t>À faire</t>
+      <c r="F98" s="33" t="inlineStr">
+        <is>
+          <t>✅ Réalisé</t>
+        </is>
+      </c>
+      <c r="G98" s="34" t="inlineStr">
+        <is>
+          <t>Itération 4</t>
         </is>
       </c>
     </row>
@@ -4337,9 +4387,14 @@
           <t>Haute</t>
         </is>
       </c>
-      <c r="F99" s="2" t="inlineStr">
-        <is>
-          <t>À faire</t>
+      <c r="F99" s="33" t="inlineStr">
+        <is>
+          <t>✅ Réalisé</t>
+        </is>
+      </c>
+      <c r="G99" s="34" t="inlineStr">
+        <is>
+          <t>Itération 4</t>
         </is>
       </c>
     </row>
@@ -4367,9 +4422,14 @@
           <t>Haute</t>
         </is>
       </c>
-      <c r="F100" s="2" t="inlineStr">
-        <is>
-          <t>À faire</t>
+      <c r="F100" s="33" t="inlineStr">
+        <is>
+          <t>✅ Réalisé</t>
+        </is>
+      </c>
+      <c r="G100" s="34" t="inlineStr">
+        <is>
+          <t>Itération 4</t>
         </is>
       </c>
     </row>
@@ -4397,9 +4457,14 @@
           <t>Haute</t>
         </is>
       </c>
-      <c r="F101" s="2" t="inlineStr">
-        <is>
-          <t>À faire</t>
+      <c r="F101" s="33" t="inlineStr">
+        <is>
+          <t>✅ Réalisé</t>
+        </is>
+      </c>
+      <c r="G101" s="34" t="inlineStr">
+        <is>
+          <t>Itération 4 — détour avec retour au checkout</t>
         </is>
       </c>
     </row>
@@ -4457,9 +4522,14 @@
           <t>Haute</t>
         </is>
       </c>
-      <c r="F103" s="2" t="inlineStr">
-        <is>
-          <t>À faire</t>
+      <c r="F103" s="35" t="inlineStr">
+        <is>
+          <t>🟡 Partiel</t>
+        </is>
+      </c>
+      <c r="G103" s="34" t="inlineStr">
+        <is>
+          <t>Forfait 1 000 FCFA/vendeur ; vrai calcul au module Livraison</t>
         </is>
       </c>
     </row>
@@ -4487,9 +4557,14 @@
           <t>Haute</t>
         </is>
       </c>
-      <c r="F104" s="2" t="inlineStr">
-        <is>
-          <t>À faire</t>
+      <c r="F104" s="35" t="inlineStr">
+        <is>
+          <t>🟡 Partiel</t>
+        </is>
+      </c>
+      <c r="G104" s="34" t="inlineStr">
+        <is>
+          <t>Affiché ; paiement actif à l'itération 5 (Escrow)</t>
         </is>
       </c>
     </row>
@@ -4517,9 +4592,14 @@
           <t>Haute</t>
         </is>
       </c>
-      <c r="F105" s="2" t="inlineStr">
-        <is>
-          <t>À faire</t>
+      <c r="F105" s="33" t="inlineStr">
+        <is>
+          <t>✅ Réalisé</t>
+        </is>
+      </c>
+      <c r="G105" s="34" t="inlineStr">
+        <is>
+          <t>Itération 4</t>
         </is>
       </c>
     </row>
@@ -4547,9 +4627,14 @@
           <t>Haute</t>
         </is>
       </c>
-      <c r="F106" s="2" t="inlineStr">
-        <is>
-          <t>À faire</t>
+      <c r="F106" s="33" t="inlineStr">
+        <is>
+          <t>✅ Réalisé</t>
+        </is>
+      </c>
+      <c r="G106" s="34" t="inlineStr">
+        <is>
+          <t>Itération 4 — statut en attente de paiement</t>
         </is>
       </c>
     </row>
@@ -4577,9 +4662,14 @@
           <t>Haute</t>
         </is>
       </c>
-      <c r="F107" s="2" t="inlineStr">
-        <is>
-          <t>À faire</t>
+      <c r="F107" s="33" t="inlineStr">
+        <is>
+          <t>✅ Réalisé</t>
+        </is>
+      </c>
+      <c r="G107" s="34" t="inlineStr">
+        <is>
+          <t>Itération 4 — format GK-AAMMJJ-XXXX</t>
         </is>
       </c>
     </row>
@@ -4607,9 +4697,14 @@
           <t>Haute</t>
         </is>
       </c>
-      <c r="F108" s="2" t="inlineStr">
-        <is>
-          <t>À faire</t>
+      <c r="F108" s="33" t="inlineStr">
+        <is>
+          <t>✅ Réalisé</t>
+        </is>
+      </c>
+      <c r="G108" s="34" t="inlineStr">
+        <is>
+          <t>Itération 4</t>
         </is>
       </c>
     </row>
@@ -4637,9 +4732,14 @@
           <t>Haute</t>
         </is>
       </c>
-      <c r="F109" s="2" t="inlineStr">
-        <is>
-          <t>À faire</t>
+      <c r="F109" s="33" t="inlineStr">
+        <is>
+          <t>✅ Réalisé</t>
+        </is>
+      </c>
+      <c r="G109" s="34" t="inlineStr">
+        <is>
+          <t>Itération 4 — une commande par vendeur, groupées</t>
         </is>
       </c>
     </row>
@@ -4667,9 +4767,14 @@
           <t>Haute</t>
         </is>
       </c>
-      <c r="F110" s="2" t="inlineStr">
-        <is>
-          <t>À faire</t>
+      <c r="F110" s="33" t="inlineStr">
+        <is>
+          <t>✅ Réalisé</t>
+        </is>
+      </c>
+      <c r="G110" s="34" t="inlineStr">
+        <is>
+          <t>Itération 4</t>
         </is>
       </c>
     </row>
@@ -4697,9 +4802,14 @@
           <t>Haute</t>
         </is>
       </c>
-      <c r="F111" s="2" t="inlineStr">
-        <is>
-          <t>À faire</t>
+      <c r="F111" s="33" t="inlineStr">
+        <is>
+          <t>✅ Réalisé</t>
+        </is>
+      </c>
+      <c r="G111" s="34" t="inlineStr">
+        <is>
+          <t>Itération 4 — prix de gros auto + qté min commande</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Suivi : iteration 8 marquee dans l explosion du projet
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Explosion du projet - MAJ.xlsx
+++ b/docs/Explosion du projet - MAJ.xlsx
@@ -1879,9 +1879,14 @@
           <t>Haute</t>
         </is>
       </c>
-      <c r="F22" s="2" t="inlineStr">
-        <is>
-          <t>À faire</t>
+      <c r="F22" s="33" t="inlineStr">
+        <is>
+          <t>✅ Réalisé</t>
+        </is>
+      </c>
+      <c r="G22" s="34" t="inlineStr">
+        <is>
+          <t>Itération 7-8 — litiges suivis depuis les commandes ; vue admin dédiée</t>
         </is>
       </c>
     </row>
@@ -8350,9 +8355,14 @@
           <t>Haute</t>
         </is>
       </c>
-      <c r="F220" s="2" t="inlineStr">
-        <is>
-          <t>À faire</t>
+      <c r="F220" s="35" t="inlineStr">
+        <is>
+          <t>🟡 Partiel</t>
+        </is>
+      </c>
+      <c r="G220" s="34" t="inlineStr">
+        <is>
+          <t>Suspension/bannissement opérationnels ; avertissement formel au module Communication</t>
         </is>
       </c>
     </row>
@@ -8380,9 +8390,14 @@
           <t>Haute</t>
         </is>
       </c>
-      <c r="F221" s="2" t="inlineStr">
-        <is>
-          <t>À faire</t>
+      <c r="F221" s="33" t="inlineStr">
+        <is>
+          <t>✅ Réalisé</t>
+        </is>
+      </c>
+      <c r="G221" s="34" t="inlineStr">
+        <is>
+          <t>Itération 8 — suspension compte et/ou boutique, réversible</t>
         </is>
       </c>
     </row>
@@ -8410,9 +8425,14 @@
           <t>Haute</t>
         </is>
       </c>
-      <c r="F222" s="2" t="inlineStr">
-        <is>
-          <t>À faire</t>
+      <c r="F222" s="33" t="inlineStr">
+        <is>
+          <t>✅ Réalisé</t>
+        </is>
+      </c>
+      <c r="G222" s="34" t="inlineStr">
+        <is>
+          <t>Itération 8 — bannissement définitif</t>
         </is>
       </c>
     </row>
@@ -8896,9 +8916,14 @@
           <t>Haute</t>
         </is>
       </c>
-      <c r="F239" s="2" t="inlineStr">
-        <is>
-          <t>À faire</t>
+      <c r="F239" s="33" t="inlineStr">
+        <is>
+          <t>✅ Réalisé</t>
+        </is>
+      </c>
+      <c r="G239" s="34" t="inlineStr">
+        <is>
+          <t>Itération 8 — dashboard /admin</t>
         </is>
       </c>
     </row>
@@ -8926,9 +8951,14 @@
           <t>Haute</t>
         </is>
       </c>
-      <c r="F240" s="2" t="inlineStr">
-        <is>
-          <t>À faire</t>
+      <c r="F240" s="33" t="inlineStr">
+        <is>
+          <t>✅ Réalisé</t>
+        </is>
+      </c>
+      <c r="G240" s="34" t="inlineStr">
+        <is>
+          <t>Itération 8 — KPIs calculés en direct sur la base</t>
         </is>
       </c>
     </row>
@@ -8956,9 +8986,14 @@
           <t>Haute</t>
         </is>
       </c>
-      <c r="F241" s="2" t="inlineStr">
-        <is>
-          <t>À faire</t>
+      <c r="F241" s="35" t="inlineStr">
+        <is>
+          <t>🟡 Partiel</t>
+        </is>
+      </c>
+      <c r="G241" s="34" t="inlineStr">
+        <is>
+          <t>KPIs chiffrés ; graphiques à venir</t>
         </is>
       </c>
     </row>
@@ -8986,9 +9021,14 @@
           <t>Moyenne</t>
         </is>
       </c>
-      <c r="F242" s="2" t="inlineStr">
-        <is>
-          <t>À faire</t>
+      <c r="F242" s="35" t="inlineStr">
+        <is>
+          <t>🟡 Partiel</t>
+        </is>
+      </c>
+      <c r="G242" s="34" t="inlineStr">
+        <is>
+          <t>KPIs chiffrés ; graphiques à venir</t>
         </is>
       </c>
     </row>
@@ -9016,9 +9056,14 @@
           <t>Haute</t>
         </is>
       </c>
-      <c r="F243" s="2" t="inlineStr">
-        <is>
-          <t>À faire</t>
+      <c r="F243" s="33" t="inlineStr">
+        <is>
+          <t>✅ Réalisé</t>
+        </is>
+      </c>
+      <c r="G243" s="34" t="inlineStr">
+        <is>
+          <t>Itération 8 — tâches en attente mises en avant</t>
         </is>
       </c>
     </row>
@@ -9046,9 +9091,14 @@
           <t>Haute</t>
         </is>
       </c>
-      <c r="F244" s="2" t="inlineStr">
-        <is>
-          <t>À faire</t>
+      <c r="F244" s="33" t="inlineStr">
+        <is>
+          <t>✅ Réalisé</t>
+        </is>
+      </c>
+      <c r="G244" s="34" t="inlineStr">
+        <is>
+          <t>Itération 8 — validations et litiges avec liens directs</t>
         </is>
       </c>
     </row>
@@ -9076,9 +9126,14 @@
           <t>Haute</t>
         </is>
       </c>
-      <c r="F245" s="2" t="inlineStr">
-        <is>
-          <t>À faire</t>
+      <c r="F245" s="33" t="inlineStr">
+        <is>
+          <t>✅ Réalisé</t>
+        </is>
+      </c>
+      <c r="G245" s="34" t="inlineStr">
+        <is>
+          <t>Itération 8 — commissions, Escrow, passif wallets</t>
         </is>
       </c>
     </row>
@@ -9106,9 +9161,14 @@
           <t>Haute</t>
         </is>
       </c>
-      <c r="F246" s="2" t="inlineStr">
-        <is>
-          <t>À faire</t>
+      <c r="F246" s="33" t="inlineStr">
+        <is>
+          <t>✅ Réalisé</t>
+        </is>
+      </c>
+      <c r="G246" s="34" t="inlineStr">
+        <is>
+          <t>Itération 8 — /admin/utilisateurs (100 derniers, recherche)</t>
         </is>
       </c>
     </row>
@@ -9136,9 +9196,14 @@
           <t>Haute</t>
         </is>
       </c>
-      <c r="F247" s="2" t="inlineStr">
-        <is>
-          <t>À faire</t>
+      <c r="F247" s="33" t="inlineStr">
+        <is>
+          <t>✅ Réalisé</t>
+        </is>
+      </c>
+      <c r="G247" s="34" t="inlineStr">
+        <is>
+          <t>Itération 8 — nom, email, téléphone + filtre statut</t>
         </is>
       </c>
     </row>
@@ -9166,9 +9231,14 @@
           <t>Haute</t>
         </is>
       </c>
-      <c r="F248" s="2" t="inlineStr">
-        <is>
-          <t>À faire</t>
+      <c r="F248" s="35" t="inlineStr">
+        <is>
+          <t>🟡 Partiel</t>
+        </is>
+      </c>
+      <c r="G248" s="34" t="inlineStr">
+        <is>
+          <t>Casquettes et statuts dans la liste ; fiche détaillée à venir</t>
         </is>
       </c>
     </row>
@@ -9196,9 +9266,14 @@
           <t>Haute</t>
         </is>
       </c>
-      <c r="F249" s="2" t="inlineStr">
-        <is>
-          <t>À faire</t>
+      <c r="F249" s="35" t="inlineStr">
+        <is>
+          <t>🟡 Partiel</t>
+        </is>
+      </c>
+      <c r="G249" s="34" t="inlineStr">
+        <is>
+          <t>Statut modifiable ; édition des informations à venir</t>
         </is>
       </c>
     </row>
@@ -9226,9 +9301,14 @@
           <t>Haute</t>
         </is>
       </c>
-      <c r="F250" s="2" t="inlineStr">
-        <is>
-          <t>À faire</t>
+      <c r="F250" s="33" t="inlineStr">
+        <is>
+          <t>✅ Réalisé</t>
+        </is>
+      </c>
+      <c r="G250" s="34" t="inlineStr">
+        <is>
+          <t>Itération 8 — session inopérante immédiatement</t>
         </is>
       </c>
     </row>
@@ -9256,9 +9336,14 @@
           <t>Haute</t>
         </is>
       </c>
-      <c r="F251" s="2" t="inlineStr">
-        <is>
-          <t>À faire</t>
+      <c r="F251" s="33" t="inlineStr">
+        <is>
+          <t>✅ Réalisé</t>
+        </is>
+      </c>
+      <c r="G251" s="34" t="inlineStr">
+        <is>
+          <t>Itération 8</t>
         </is>
       </c>
     </row>
@@ -9286,9 +9371,14 @@
           <t>Haute</t>
         </is>
       </c>
-      <c r="F252" s="2" t="inlineStr">
-        <is>
-          <t>À faire</t>
+      <c r="F252" s="33" t="inlineStr">
+        <is>
+          <t>✅ Réalisé</t>
+        </is>
+      </c>
+      <c r="G252" s="34" t="inlineStr">
+        <is>
+          <t>Itération 2 — file de validation avec documents KYC</t>
         </is>
       </c>
     </row>
@@ -9316,9 +9406,14 @@
           <t>Haute</t>
         </is>
       </c>
-      <c r="F253" s="2" t="inlineStr">
-        <is>
-          <t>À faire</t>
+      <c r="F253" s="33" t="inlineStr">
+        <is>
+          <t>✅ Réalisé</t>
+        </is>
+      </c>
+      <c r="G253" s="34" t="inlineStr">
+        <is>
+          <t>Itérations 2-8 — toutes les demandes et boutiques listées</t>
         </is>
       </c>
     </row>
@@ -9346,9 +9441,14 @@
           <t>Haute</t>
         </is>
       </c>
-      <c r="F254" s="2" t="inlineStr">
-        <is>
-          <t>À faire</t>
+      <c r="F254" s="35" t="inlineStr">
+        <is>
+          <t>🟡 Partiel</t>
+        </is>
+      </c>
+      <c r="G254" s="34" t="inlineStr">
+        <is>
+          <t>Visible via dashboard et financier ; fiche vendeur à venir</t>
         </is>
       </c>
     </row>
@@ -9406,9 +9506,14 @@
           <t>Haute</t>
         </is>
       </c>
-      <c r="F256" s="2" t="inlineStr">
-        <is>
-          <t>À faire</t>
+      <c r="F256" s="33" t="inlineStr">
+        <is>
+          <t>✅ Réalisé</t>
+        </is>
+      </c>
+      <c r="G256" s="34" t="inlineStr">
+        <is>
+          <t>Itération 8 — produits retirés de tout le parcours public</t>
         </is>
       </c>
     </row>
@@ -9436,9 +9541,14 @@
           <t>Haute</t>
         </is>
       </c>
-      <c r="F257" s="2" t="inlineStr">
-        <is>
-          <t>À faire</t>
+      <c r="F257" s="35" t="inlineStr">
+        <is>
+          <t>🟡 Partiel</t>
+        </is>
+      </c>
+      <c r="G257" s="34" t="inlineStr">
+        <is>
+          <t>Suspension réversible ; fermeture définitive = suspension + bannissement</t>
         </is>
       </c>
     </row>
@@ -9466,9 +9576,14 @@
           <t>Haute</t>
         </is>
       </c>
-      <c r="F258" s="2" t="inlineStr">
-        <is>
-          <t>À faire</t>
+      <c r="F258" s="33" t="inlineStr">
+        <is>
+          <t>✅ Réalisé</t>
+        </is>
+      </c>
+      <c r="G258" s="34" t="inlineStr">
+        <is>
+          <t>Itération 8 — /admin/produits (recherche + filtre statut)</t>
         </is>
       </c>
     </row>
@@ -9496,9 +9611,14 @@
           <t>Haute</t>
         </is>
       </c>
-      <c r="F259" s="2" t="inlineStr">
-        <is>
-          <t>À faire</t>
+      <c r="F259" s="35" t="inlineStr">
+        <is>
+          <t>🟡 Partiel</t>
+        </is>
+      </c>
+      <c r="G259" s="34" t="inlineStr">
+        <is>
+          <t>Modération a posteriori ; pré-modération des nouveautés à venir</t>
         </is>
       </c>
     </row>
@@ -9526,9 +9646,14 @@
           <t>Haute</t>
         </is>
       </c>
-      <c r="F260" s="2" t="inlineStr">
-        <is>
-          <t>À faire</t>
+      <c r="F260" s="35" t="inlineStr">
+        <is>
+          <t>🟡 Partiel</t>
+        </is>
+      </c>
+      <c r="G260" s="34" t="inlineStr">
+        <is>
+          <t>Retrait/republication ; édition directe à venir</t>
         </is>
       </c>
     </row>
@@ -9556,9 +9681,14 @@
           <t>Haute</t>
         </is>
       </c>
-      <c r="F261" s="2" t="inlineStr">
-        <is>
-          <t>À faire</t>
+      <c r="F261" s="33" t="inlineStr">
+        <is>
+          <t>✅ Réalisé</t>
+        </is>
+      </c>
+      <c r="G261" s="34" t="inlineStr">
+        <is>
+          <t>Itération 8 — archivage de modération (le vendeur peut corriger)</t>
         </is>
       </c>
     </row>
@@ -9586,9 +9716,14 @@
           <t>Haute</t>
         </is>
       </c>
-      <c r="F262" s="2" t="inlineStr">
-        <is>
-          <t>À faire</t>
+      <c r="F262" s="33" t="inlineStr">
+        <is>
+          <t>✅ Réalisé</t>
+        </is>
+      </c>
+      <c r="G262" s="34" t="inlineStr">
+        <is>
+          <t>Itération 8 — retrait du catalogue immédiat</t>
         </is>
       </c>
     </row>
@@ -9616,9 +9751,14 @@
           <t>Haute</t>
         </is>
       </c>
-      <c r="F263" s="2" t="inlineStr">
-        <is>
-          <t>À faire</t>
+      <c r="F263" s="33" t="inlineStr">
+        <is>
+          <t>✅ Réalisé</t>
+        </is>
+      </c>
+      <c r="G263" s="34" t="inlineStr">
+        <is>
+          <t>Itération 8 — /admin/commandes</t>
         </is>
       </c>
     </row>
@@ -9646,9 +9786,14 @@
           <t>Haute</t>
         </is>
       </c>
-      <c r="F264" s="2" t="inlineStr">
-        <is>
-          <t>À faire</t>
+      <c r="F264" s="35" t="inlineStr">
+        <is>
+          <t>🟡 Partiel</t>
+        </is>
+      </c>
+      <c r="G264" s="34" t="inlineStr">
+        <is>
+          <t>Filtre statut + recherche n° ; filtres avancés à venir</t>
         </is>
       </c>
     </row>
@@ -9676,9 +9821,14 @@
           <t>Haute</t>
         </is>
       </c>
-      <c r="F265" s="2" t="inlineStr">
-        <is>
-          <t>À faire</t>
+      <c r="F265" s="33" t="inlineStr">
+        <is>
+          <t>✅ Réalisé</t>
+        </is>
+      </c>
+      <c r="G265" s="34" t="inlineStr">
+        <is>
+          <t>Itération 8 — acheteur, boutique, montants, commission</t>
         </is>
       </c>
     </row>
@@ -9706,9 +9856,14 @@
           <t>Haute</t>
         </is>
       </c>
-      <c r="F266" s="2" t="inlineStr">
-        <is>
-          <t>À faire</t>
+      <c r="F266" s="35" t="inlineStr">
+        <is>
+          <t>🟡 Partiel</t>
+        </is>
+      </c>
+      <c r="G266" s="34" t="inlineStr">
+        <is>
+          <t>Annulation manuelle ; autres transitions forcées à venir</t>
         </is>
       </c>
     </row>
@@ -9736,9 +9891,14 @@
           <t>Haute</t>
         </is>
       </c>
-      <c r="F267" s="2" t="inlineStr">
-        <is>
-          <t>À faire</t>
+      <c r="F267" s="33" t="inlineStr">
+        <is>
+          <t>✅ Réalisé</t>
+        </is>
+      </c>
+      <c r="G267" s="34" t="inlineStr">
+        <is>
+          <t>Itération 8 — avec re-stock et annulation des courses</t>
         </is>
       </c>
     </row>
@@ -9766,9 +9926,14 @@
           <t>Haute</t>
         </is>
       </c>
-      <c r="F268" s="2" t="inlineStr">
-        <is>
-          <t>À faire</t>
+      <c r="F268" s="33" t="inlineStr">
+        <is>
+          <t>✅ Réalisé</t>
+        </is>
+      </c>
+      <c r="G268" s="34" t="inlineStr">
+        <is>
+          <t>Itération 8 — remboursement wallet intégral si payée</t>
         </is>
       </c>
     </row>
@@ -9796,9 +9961,14 @@
           <t>Haute</t>
         </is>
       </c>
-      <c r="F269" s="2" t="inlineStr">
-        <is>
-          <t>À faire</t>
+      <c r="F269" s="33" t="inlineStr">
+        <is>
+          <t>✅ Réalisé</t>
+        </is>
+      </c>
+      <c r="G269" s="34" t="inlineStr">
+        <is>
+          <t>Itération 8 — /admin/financier</t>
         </is>
       </c>
     </row>
@@ -9826,9 +9996,14 @@
           <t>Haute</t>
         </is>
       </c>
-      <c r="F270" s="2" t="inlineStr">
-        <is>
-          <t>À faire</t>
+      <c r="F270" s="33" t="inlineStr">
+        <is>
+          <t>✅ Réalisé</t>
+        </is>
+      </c>
+      <c r="G270" s="34" t="inlineStr">
+        <is>
+          <t>Itération 8 — fonds bloqués + grand livre</t>
         </is>
       </c>
     </row>
@@ -9856,9 +10031,14 @@
           <t>Haute</t>
         </is>
       </c>
-      <c r="F271" s="2" t="inlineStr">
-        <is>
-          <t>À faire</t>
+      <c r="F271" s="33" t="inlineStr">
+        <is>
+          <t>✅ Réalisé</t>
+        </is>
+      </c>
+      <c r="G271" s="34" t="inlineStr">
+        <is>
+          <t>Itération 8 — Escrow en attente de déblocage</t>
         </is>
       </c>
     </row>
@@ -9886,9 +10066,14 @@
           <t>Haute</t>
         </is>
       </c>
-      <c r="F272" s="2" t="inlineStr">
-        <is>
-          <t>À faire</t>
+      <c r="F272" s="33" t="inlineStr">
+        <is>
+          <t>✅ Réalisé</t>
+        </is>
+      </c>
+      <c r="G272" s="34" t="inlineStr">
+        <is>
+          <t>Itération 8 — versements vendeurs/livreurs dans le grand livre</t>
         </is>
       </c>
     </row>
@@ -9916,9 +10101,14 @@
           <t>Haute</t>
         </is>
       </c>
-      <c r="F273" s="2" t="inlineStr">
-        <is>
-          <t>À faire</t>
+      <c r="F273" s="33" t="inlineStr">
+        <is>
+          <t>✅ Réalisé</t>
+        </is>
+      </c>
+      <c r="G273" s="34" t="inlineStr">
+        <is>
+          <t>Itération 8 — total remboursé + mouvements</t>
         </is>
       </c>
     </row>
@@ -9946,9 +10136,14 @@
           <t>Haute</t>
         </is>
       </c>
-      <c r="F274" s="2" t="inlineStr">
-        <is>
-          <t>À faire</t>
+      <c r="F274" s="33" t="inlineStr">
+        <is>
+          <t>✅ Réalisé</t>
+        </is>
+      </c>
+      <c r="G274" s="34" t="inlineStr">
+        <is>
+          <t>Itération 8 — total et par commande</t>
         </is>
       </c>
     </row>
@@ -9976,9 +10171,14 @@
           <t>Haute</t>
         </is>
       </c>
-      <c r="F275" s="2" t="inlineStr">
-        <is>
-          <t>À faire</t>
+      <c r="F275" s="35" t="inlineStr">
+        <is>
+          <t>🟡 Partiel</t>
+        </is>
+      </c>
+      <c r="G275" s="34" t="inlineStr">
+        <is>
+          <t>Indicateurs en ligne ; exports comptables à venir</t>
         </is>
       </c>
     </row>
@@ -10426,9 +10626,14 @@
           <t>Haute</t>
         </is>
       </c>
-      <c r="F290" s="2" t="inlineStr">
-        <is>
-          <t>À faire</t>
+      <c r="F290" s="35" t="inlineStr">
+        <is>
+          <t>🟡 Partiel</t>
+        </is>
+      </c>
+      <c r="G290" s="34" t="inlineStr">
+        <is>
+          <t>Produits non conformes retirables ; signalements utilisateurs à venir</t>
         </is>
       </c>
     </row>
@@ -10456,9 +10661,14 @@
           <t>Haute</t>
         </is>
       </c>
-      <c r="F291" s="2" t="inlineStr">
-        <is>
-          <t>À faire</t>
+      <c r="F291" s="33" t="inlineStr">
+        <is>
+          <t>✅ Réalisé</t>
+        </is>
+      </c>
+      <c r="G291" s="34" t="inlineStr">
+        <is>
+          <t>Itération 8 — retrait produit, suspension boutique/compte</t>
         </is>
       </c>
     </row>
@@ -10708,9 +10918,14 @@
           <t>Haute</t>
         </is>
       </c>
-      <c r="F300" s="2" t="inlineStr">
-        <is>
-          <t>À faire</t>
+      <c r="F300" s="33" t="inlineStr">
+        <is>
+          <t>✅ Réalisé</t>
+        </is>
+      </c>
+      <c r="G300" s="34" t="inlineStr">
+        <is>
+          <t>Itération 5 — 5 % calculés au versement</t>
         </is>
       </c>
     </row>
@@ -10738,9 +10953,14 @@
           <t>Haute</t>
         </is>
       </c>
-      <c r="F301" s="2" t="inlineStr">
-        <is>
-          <t>À faire</t>
+      <c r="F301" s="33" t="inlineStr">
+        <is>
+          <t>✅ Réalisé</t>
+        </is>
+      </c>
+      <c r="G301" s="34" t="inlineStr">
+        <is>
+          <t>Itération 5 — prélevée sur le versement vendeur</t>
         </is>
       </c>
     </row>
@@ -10768,9 +10988,14 @@
           <t>Haute</t>
         </is>
       </c>
-      <c r="F302" s="2" t="inlineStr">
-        <is>
-          <t>À faire</t>
+      <c r="F302" s="33" t="inlineStr">
+        <is>
+          <t>✅ Réalisé</t>
+        </is>
+      </c>
+      <c r="G302" s="34" t="inlineStr">
+        <is>
+          <t>Itération 8 — commission par commande + total plateforme</t>
         </is>
       </c>
     </row>
@@ -10930,9 +11155,14 @@
           <t>Haute</t>
         </is>
       </c>
-      <c r="F308" s="2" t="inlineStr">
-        <is>
-          <t>À faire</t>
+      <c r="F308" s="33" t="inlineStr">
+        <is>
+          <t>✅ Réalisé</t>
+        </is>
+      </c>
+      <c r="G308" s="34" t="inlineStr">
+        <is>
+          <t>Itérations 1-8 — Tailwind responsive sur tout le parcours</t>
         </is>
       </c>
     </row>
@@ -11122,9 +11352,14 @@
           <t>Haute</t>
         </is>
       </c>
-      <c r="F315" s="2" t="inlineStr">
-        <is>
-          <t>À faire</t>
+      <c r="F315" s="33" t="inlineStr">
+        <is>
+          <t>✅ Réalisé</t>
+        </is>
+      </c>
+      <c r="G315" s="34" t="inlineStr">
+        <is>
+          <t>Itération 8</t>
         </is>
       </c>
     </row>
@@ -11152,9 +11387,14 @@
           <t>Haute</t>
         </is>
       </c>
-      <c r="F316" s="2" t="inlineStr">
-        <is>
-          <t>À faire</t>
+      <c r="F316" s="33" t="inlineStr">
+        <is>
+          <t>✅ Réalisé</t>
+        </is>
+      </c>
+      <c r="G316" s="34" t="inlineStr">
+        <is>
+          <t>Itération 8</t>
         </is>
       </c>
     </row>
@@ -11182,9 +11422,14 @@
           <t>Haute</t>
         </is>
       </c>
-      <c r="F317" s="2" t="inlineStr">
-        <is>
-          <t>À faire</t>
+      <c r="F317" s="33" t="inlineStr">
+        <is>
+          <t>✅ Réalisé</t>
+        </is>
+      </c>
+      <c r="G317" s="34" t="inlineStr">
+        <is>
+          <t>Itération 8</t>
         </is>
       </c>
     </row>
@@ -11212,9 +11457,14 @@
           <t>Haute</t>
         </is>
       </c>
-      <c r="F318" s="2" t="inlineStr">
-        <is>
-          <t>À faire</t>
+      <c r="F318" s="33" t="inlineStr">
+        <is>
+          <t>✅ Réalisé</t>
+        </is>
+      </c>
+      <c r="G318" s="34" t="inlineStr">
+        <is>
+          <t>Itération 8</t>
         </is>
       </c>
     </row>

</xml_diff>